<commit_message>
Add ICDC number and invoice date to excel uploads and fix date formatting
Update Excel parsing to capture "ICDC Number" and "Invoice Date", normalize column headers, and correctly format Excel date serials.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 07fac953-cb09-45b9-a059-9c9e1d332a82
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 08346c72-16de-4e38-848e-217f3451acf1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/19da168d-5ad0-4818-a3b9-67bbf1ae28cd/07fac953-cb09-45b9-a059-9c9e1d332a82/mOHWPhB
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/Invoice_Template_1775231757722.xlsx
+++ b/attached_assets/Invoice_Template_1775231757722.xlsx
@@ -1,128 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F16C89C-2A64-4D4E-A255-EBBAC14AEC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Invoice Template" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
-  <si>
-    <t>Sl.No.</t>
-  </si>
-  <si>
-    <t>Brand Number</t>
-  </si>
-  <si>
-    <t>Brand Name</t>
-  </si>
-  <si>
-    <t>Product Type</t>
-  </si>
-  <si>
-    <t>Pack Type</t>
-  </si>
-  <si>
-    <t>Pack Qty / Size (ml)</t>
-  </si>
-  <si>
-    <t>Qty Cases Delivered</t>
-  </si>
-  <si>
-    <t>Qty Bottles Delivered</t>
-  </si>
-  <si>
-    <t>Rate Per Case</t>
-  </si>
-  <si>
-    <t>Unit Rate Per Bottle</t>
-  </si>
-  <si>
-    <t>Total Amount</t>
-  </si>
-  <si>
-    <t>Breakage Btl Qty</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>5029</t>
-  </si>
-  <si>
-    <t>KINGFISHER ULTRA LAGER BEER</t>
-  </si>
-  <si>
-    <t>Beer</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>12 / 650 ml</t>
-  </si>
-  <si>
-    <t>2201.00</t>
-  </si>
-  <si>
-    <t>183.42</t>
-  </si>
-  <si>
-    <t>48422.00</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>0110</t>
-  </si>
-  <si>
-    <t>OFFICER'S CHOICE RESERVE WHISKY</t>
-  </si>
-  <si>
-    <t>IML</t>
-  </si>
-  <si>
-    <t>48 / 180 ml</t>
-  </si>
-  <si>
-    <t>5204.00</t>
-  </si>
-  <si>
-    <t>108.42</t>
-  </si>
-  <si>
-    <t>156011.58</t>
-  </si>
-  <si>
-    <t>ICDC Number</t>
-  </si>
-  <si>
-    <t>Invoice Date:</t>
-  </si>
-  <si>
-    <t>ICDC019050226013418</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -151,23 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -492,98 +396,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6.875" customWidth="1"/>
-    <col min="2" max="2" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.875" customWidth="1"/>
-    <col min="5" max="5" width="45.875" customWidth="1"/>
-    <col min="6" max="6" width="14.875" customWidth="1"/>
-    <col min="7" max="7" width="10.875" customWidth="1"/>
-    <col min="8" max="8" width="20.875" customWidth="1"/>
-    <col min="9" max="9" width="18.875" customWidth="1"/>
-    <col min="10" max="10" width="20.875" customWidth="1"/>
-    <col min="11" max="11" width="14.875" customWidth="1"/>
-    <col min="12" max="12" width="20.875" customWidth="1"/>
-    <col min="13" max="13" width="14.875" customWidth="1"/>
-    <col min="14" max="14" width="16.875" customWidth="1"/>
-    <col min="15" max="15" width="15.875" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" t="s">
-        <v>12</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Sl.No.</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ICDC Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Invoice Date</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Brand Number</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Brand Name</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Product Type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Pack Type</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Pack Qty / Size (ml)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Qty Cases Delivered</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Qty Bottles Delivered</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Rate Per Case</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Unit Rate Per Bottle</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Total Amount</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Breakage Btl Qty</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Remarks</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B2" t="str">
+        <v>ICDC019050226013418</v>
+      </c>
+      <c r="C2">
         <v>46058</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>17</v>
+      <c r="D2" t="str">
+        <v>5029</v>
+      </c>
+      <c r="E2" t="str">
+        <v>KINGFISHER ULTRA LAGER BEER</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Beer</v>
+      </c>
+      <c r="G2" t="str">
+        <v>G</v>
+      </c>
+      <c r="H2" t="str">
+        <v>12 / 650 ml</v>
       </c>
       <c r="I2">
         <v>22</v>
@@ -591,46 +477,46 @@
       <c r="J2">
         <v>0</v>
       </c>
-      <c r="K2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" t="s">
-        <v>20</v>
+      <c r="K2" t="str">
+        <v>2201.00</v>
+      </c>
+      <c r="L2" t="str">
+        <v>183.42</v>
+      </c>
+      <c r="M2" t="str">
+        <v>48422.00</v>
       </c>
       <c r="N2">
         <v>0</v>
       </c>
-      <c r="O2" t="s">
-        <v>21</v>
+      <c r="O2" t="str">
+        <v/>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3" t="str">
+        <v>ICDC019050226013418</v>
+      </c>
+      <c r="C3">
         <v>46058</v>
       </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" t="s">
-        <v>25</v>
+      <c r="D3" t="str">
+        <v>0110</v>
+      </c>
+      <c r="E3" t="str">
+        <v>OFFICER'S CHOICE RESERVE WHISKY</v>
+      </c>
+      <c r="F3" t="str">
+        <v>IML</v>
+      </c>
+      <c r="G3" t="str">
+        <v>G</v>
+      </c>
+      <c r="H3" t="str">
+        <v>48 / 180 ml</v>
       </c>
       <c r="I3">
         <v>29</v>
@@ -638,26 +524,26 @@
       <c r="J3">
         <v>47</v>
       </c>
-      <c r="K3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M3" t="s">
-        <v>28</v>
+      <c r="K3" t="str">
+        <v>5204.00</v>
+      </c>
+      <c r="L3" t="str">
+        <v>108.42</v>
+      </c>
+      <c r="M3" t="str">
+        <v>156011.58</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
-      <c r="O3" t="s">
-        <v>21</v>
+      <c r="O3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="D1:O3 A1:A3" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>